<commit_message>
fixed borders on nested-style files
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/schedule/DaySchedule.xlsx
+++ b/owlcms/src/main/resources/templates/schedule/DaySchedule.xlsx
@@ -54,7 +54,9 @@
             <family val="2"/>
           </rPr>
           <t>jx:area(lastCell="L5")
-owlcms:fixMerges(5, [1, 2, 3])</t>
+owlcms:mergeDown(5, 1, 3)
+owlcms:horizontalBorders(5, 1, 3)
+owlcms:verticalBorders(5, 1, 12)</t>
         </r>
       </text>
     </comment>
@@ -90,8 +92,7 @@
   var="sessionBlock"
   groupBy="sessionBlock.sessionBlock"
   lastCell="L5"
-)
-owlcms:mergeDown</t>
+)</t>
         </r>
       </text>
     </comment>

</xml_diff>